<commit_message>
feat(calibration, maintenance): add asset image handling and display in PDF exports
- Implemented functionality to fetch and encode asset images as base64 for calibration and maintenance detail PDFs.
- Enhanced error handling for image retrieval, ensuring graceful degradation if image fetching fails.
- Updated PDF templates to display asset images, improving visual representation of asset information.
- Added checks for asset image paths and fallback mechanisms to ensure robust image handling in reports.
</commit_message>
<xml_diff>
--- a/public/docs/ImportAsetTemplate.xlsx
+++ b/public/docs/ImportAsetTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fauza\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\Collage\magang\ExcelTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30BAAD1B-5D4A-4B38-9C8B-B9326CD6DB50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F260AC3F-7C43-41A3-9407-92127045F0BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1848" yWindow="1848" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Aset" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
   <si>
     <t>nama kolom</t>
   </si>
@@ -637,14 +637,14 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -926,24 +926,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.33203125" customWidth="1"/>
     <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.88671875" customWidth="1"/>
-    <col min="10" max="10" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.88671875" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -954,40 +955,43 @@
         <v>28</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="O1" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>37</v>
       </c>
@@ -997,37 +1001,40 @@
       <c r="C2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="8">
+      <c r="G2" s="8">
         <v>5000000</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="J2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="8">
+      <c r="K2" s="8">
         <v>5000000</v>
       </c>
-      <c r="K2" s="7">
+      <c r="L2" s="7">
         <v>500000</v>
       </c>
-      <c r="L2" s="7">
+      <c r="M2" s="7">
         <v>60</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="N2" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="N2" s="12">
+      <c r="O2" s="12">
         <v>1234</v>
       </c>
     </row>
@@ -1054,10 +1061,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="26"/>
+      <c r="B1" s="28"/>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
       <c r="E1" s="14"/>
@@ -1085,7 +1092,7 @@
       <c r="C3" s="20">
         <v>100</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="26" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="19" t="s">
@@ -1100,7 +1107,7 @@
       <c r="C4" s="20">
         <v>100</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="27" t="s">
         <v>27</v>
       </c>
       <c r="E4" s="19" t="s">
@@ -1115,7 +1122,7 @@
       <c r="C5" s="20">
         <v>50</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="27" t="s">
         <v>29</v>
       </c>
       <c r="E5" s="19" t="s">

</xml_diff>